<commit_message>
edit outliers, modelos, sma, Rstudio
</commit_message>
<xml_diff>
--- a/Results_isofys/data_for_R.xlsx
+++ b/Results_isofys/data_for_R.xlsx
@@ -5883,15 +5883,9 @@
       <c r="BF28" t="n">
         <v>61.80318961158282</v>
       </c>
-      <c r="BG28" t="n">
-        <v>0.3924651391362423</v>
-      </c>
-      <c r="BH28" t="n">
-        <v>157.4743421736833</v>
-      </c>
-      <c r="BI28" t="n">
-        <v>4.948132060014879</v>
-      </c>
+      <c r="BG28" t="inlineStr"/>
+      <c r="BH28" t="inlineStr"/>
+      <c r="BI28" t="inlineStr"/>
       <c r="BJ28" t="n">
         <v>0</v>
       </c>
@@ -9106,9 +9100,7 @@
       <c r="AX45" t="n">
         <v>0.4354889097157138</v>
       </c>
-      <c r="AY45" t="n">
-        <v>34.94837353504887</v>
-      </c>
+      <c r="AY45" t="inlineStr"/>
       <c r="AZ45" t="n">
         <v>-1.016944806660762</v>
       </c>
@@ -9125,15 +9117,11 @@
       <c r="BE45" t="n">
         <v>2.080347916779913</v>
       </c>
-      <c r="BF45" t="n">
-        <v>72.70477607848517</v>
-      </c>
+      <c r="BF45" t="inlineStr"/>
       <c r="BG45" t="n">
         <v>0.06832299360407701</v>
       </c>
-      <c r="BH45" t="n">
-        <v>1064.133350183688</v>
-      </c>
+      <c r="BH45" t="inlineStr"/>
       <c r="BI45" t="n">
         <v>30.44872314634313</v>
       </c>
@@ -13877,9 +13865,7 @@
       <c r="AX70" t="n">
         <v>0.5284035259549461</v>
       </c>
-      <c r="AY70" t="n">
-        <v>33.07869485466202</v>
-      </c>
+      <c r="AY70" t="inlineStr"/>
       <c r="AZ70" t="n">
         <v>-0.9735100220183867</v>
       </c>
@@ -13896,15 +13882,11 @@
       <c r="BE70" t="n">
         <v>1.653302877966243</v>
       </c>
-      <c r="BF70" t="n">
-        <v>54.68910140257988</v>
-      </c>
+      <c r="BF70" t="inlineStr"/>
       <c r="BG70" t="n">
         <v>0.06809229172210589</v>
       </c>
-      <c r="BH70" t="n">
-        <v>803.1614154767136</v>
-      </c>
+      <c r="BH70" t="inlineStr"/>
       <c r="BI70" t="n">
         <v>24.28032360422824</v>
       </c>
@@ -16358,9 +16340,7 @@
       <c r="AX83" t="n">
         <v>0.5595520868680013</v>
       </c>
-      <c r="AY83" t="n">
-        <v>26.31625012037236</v>
-      </c>
+      <c r="AY83" t="inlineStr"/>
       <c r="AZ83" t="n">
         <v>-1.045162407612312</v>
       </c>
@@ -16377,15 +16357,11 @@
       <c r="BE83" t="n">
         <v>1.574768288150041</v>
       </c>
-      <c r="BF83" t="n">
-        <v>41.44199615258708</v>
-      </c>
+      <c r="BF83" t="inlineStr"/>
       <c r="BG83" t="n">
         <v>0.09914099335271642</v>
       </c>
-      <c r="BH83" t="n">
-        <v>418.0107012358434</v>
-      </c>
+      <c r="BH83" t="inlineStr"/>
       <c r="BI83" t="n">
         <v>15.88412860205513</v>
       </c>
@@ -25782,9 +25758,7 @@
       <c r="AX131" t="n">
         <v>0.5674558436677941</v>
       </c>
-      <c r="AY131" t="n">
-        <v>40.16479905872413</v>
-      </c>
+      <c r="AY131" t="inlineStr"/>
       <c r="AZ131" t="n">
         <v>-0.9594183293878932</v>
       </c>
@@ -25801,15 +25775,11 @@
       <c r="BE131" t="n">
         <v>2.767649227576972</v>
       </c>
-      <c r="BF131" t="n">
-        <v>111.1620750906621</v>
-      </c>
+      <c r="BF131" t="inlineStr"/>
       <c r="BG131" t="n">
         <v>0.3372710106638011</v>
       </c>
-      <c r="BH131" t="n">
-        <v>329.5927357405492</v>
-      </c>
+      <c r="BH131" t="inlineStr"/>
       <c r="BI131" t="n">
         <v>8.206009826133037</v>
       </c>
@@ -26787,15 +26757,9 @@
       <c r="BF136" t="n">
         <v>129.9570950195319</v>
       </c>
-      <c r="BG136" t="n">
-        <v>0.984908331811914</v>
-      </c>
-      <c r="BH136" t="n">
-        <v>131.9484167429599</v>
-      </c>
-      <c r="BI136" t="n">
-        <v>3.003319044462487</v>
-      </c>
+      <c r="BG136" t="inlineStr"/>
+      <c r="BH136" t="inlineStr"/>
+      <c r="BI136" t="inlineStr"/>
       <c r="BJ136" t="n">
         <v>0</v>
       </c>
@@ -27157,9 +27121,7 @@
       <c r="AX138" t="n">
         <v>0.5884236453201971</v>
       </c>
-      <c r="AY138" t="n">
-        <v>56.82593529734338</v>
-      </c>
+      <c r="AY138" t="inlineStr"/>
       <c r="AZ138" t="n">
         <v>-0.8111718275652702</v>
       </c>
@@ -27176,15 +27138,11 @@
       <c r="BE138" t="n">
         <v>2.038052013688129</v>
       </c>
-      <c r="BF138" t="n">
-        <v>115.814211862462</v>
-      </c>
+      <c r="BF138" t="inlineStr"/>
       <c r="BG138" t="n">
         <v>0.1252576192118186</v>
       </c>
-      <c r="BH138" t="n">
-        <v>924.6081203779931</v>
-      </c>
+      <c r="BH138" t="inlineStr"/>
       <c r="BI138" t="n">
         <v>16.27088257395068</v>
       </c>
@@ -27746,9 +27704,7 @@
       <c r="AX141" t="n">
         <v>0.4660103141115798</v>
       </c>
-      <c r="AY141" t="n">
-        <v>16.82978356315537</v>
-      </c>
+      <c r="AY141" t="inlineStr"/>
       <c r="AZ141" t="n">
         <v>-0.8676616915422886</v>
       </c>
@@ -27762,9 +27718,7 @@
       <c r="BD141" t="n">
         <v>1.034293220205778</v>
       </c>
-      <c r="BE141" t="n">
-        <v>9.247567853121815</v>
-      </c>
+      <c r="BE141" t="inlineStr"/>
       <c r="BF141" t="n">
         <v>155.6345654536335</v>
       </c>
@@ -27774,9 +27728,7 @@
       <c r="BH141" t="n">
         <v>481.2562334709375</v>
       </c>
-      <c r="BI141" t="n">
-        <v>28.59550936380004</v>
-      </c>
+      <c r="BI141" t="inlineStr"/>
       <c r="BJ141" t="n">
         <v>0</v>
       </c>

</xml_diff>